<commit_message>
update project version 03
</commit_message>
<xml_diff>
--- a/pms/PM_Web_Application_With_FastAPI.xlsx
+++ b/pms/PM_Web_Application_With_FastAPI.xlsx
@@ -492,7 +492,6 @@
           <t>Hiểu rõ mục tiêu môn học &amp; Mô hình sản phẩm cuối khóa</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -528,7 +527,6 @@
           <t>Kế hoạch học tập cá nhân</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -564,7 +562,6 @@
           <t>Máy tính cá nhân sẵn sàng công cụ phát triển</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -597,10 +594,9 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Vẽ được sơ đồ Client → API → Database</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>Vẽ được sơ đồ Client → API → Database. Chèn trực tiếp mã &lt;svg&gt; vào trong trường solution, TUYỆT ĐỐI KHÔNG bọc mã SVG trong các khối code block như ```xml hay ```html hay bất kỳ thẻ pre/code nào để trình duyệt có thể render trực quan đồ họa.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -623,7 +619,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Lesson 02: Thiết lập môi trường và Virtual Environment</t>
+          <t>Lesson 02: Thiết lập Virtual Environment</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -636,7 +632,6 @@
           <t>Môi trường Python + FastAPI hoạt động</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -672,7 +667,6 @@
           <t>Project FastAPI đầu tiên chạy bằng Uvicorn</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -708,7 +702,6 @@
           <t>Endpoint /hello hoạt động</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -744,7 +737,6 @@
           <t>Swagger hiển thị và test được API thành công</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -780,7 +772,6 @@
           <t>Học viên hiểu rõ Swagger UI sinh ra từ đâu.</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -816,7 +807,6 @@
           <t>Có bộ khung thư mục chuẩn bị cho việc kết nối Database.</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -852,7 +842,6 @@
           <t>Cấu trúc Router phân mảnh hoạt động tốt</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -888,7 +877,6 @@
           <t>Giao diện Swagger có thông tin dự án tùy chỉnh</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -924,7 +912,6 @@
           <t>API /users/{id} hoạt động chính xác</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -960,7 +947,6 @@
           <t>API /products?name=laptop và phân trang</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -996,7 +982,6 @@
           <t>API Create User nhận JSON hợp lệ</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1032,7 +1017,6 @@
           <t>API tự động validate dữ liệu, trả về lỗi 422 nếu sai định dạng</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1068,7 +1052,6 @@
           <t>API POST thêm mới bản ghi</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1104,7 +1087,6 @@
           <t>API GET lấy dữ liệu</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1140,7 +1122,6 @@
           <t>API PUT cập nhật thông tin</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1176,7 +1157,6 @@
           <t>API DELETE xóa bản ghi thành công</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1212,7 +1192,6 @@
           <t>Mã nguồn API CRUD Sách chạy mượt mà</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1248,7 +1227,6 @@
           <t>File Collection Postman xuất ra thành công</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1284,7 +1262,6 @@
           <t>API có response_model lọc trường</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1320,7 +1297,6 @@
           <t>API trả về đúng status code tương ứng</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1356,7 +1332,6 @@
           <t>Định dạng JSON Response chuẩn hóa</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1392,7 +1367,6 @@
           <t>Global Exception Handler bắt lỗi 500</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1428,7 +1402,6 @@
           <t>Bộ API Sách trả lỗi chuẩn hóa đẹp mắt</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1464,7 +1437,6 @@
           <t>API trả lỗi 404 tùy biến thân thiện</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1500,7 +1472,6 @@
           <t>Bản thiết kế danh sách API Endpoint</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1536,7 +1507,6 @@
           <t>Contact Management API chạy trong bộ nhớ</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1572,7 +1542,6 @@
           <t>Bộ API hoạt động hoàn chỉnh, không lỗi</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1608,7 +1577,6 @@
           <t>Hiểu mapping Table ↔ Object</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1644,7 +1612,6 @@
           <t>Kết nối thành công tới Database</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1680,7 +1647,6 @@
           <t>Model User ánh xạ vào Database</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1716,7 +1682,6 @@
           <t>Service thêm và lấy dữ liệu thành công</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1752,7 +1717,6 @@
           <t>Module database kết nối tự động</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1788,7 +1752,6 @@
           <t>API GET &amp; POST làm việc trực tiếp với MySQL</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1824,7 +1787,6 @@
           <t>Service Update hoàn thành</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1860,7 +1822,6 @@
           <t>Service Delete hoàn thành</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1896,7 +1857,6 @@
           <t>Model + Schema hoạt động đồng bộ</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1932,7 +1892,6 @@
           <t>Dependency get_db tối ưu</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1968,7 +1927,6 @@
           <t>Hệ thống quản lý sách lưu trữ bền vững</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2004,7 +1962,6 @@
           <t>API GET list phân trang hoạt động tốt</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2040,7 +1997,6 @@
           <t>Hiểu kiến trúc dự án chuẩn</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2076,7 +2032,6 @@
           <t>Module routers tách biệt</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2112,7 +2067,6 @@
           <t>Module schemas tập trung</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2148,7 +2102,6 @@
           <t>Module models tập trung</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2184,7 +2137,6 @@
           <t>Module services tập trung</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2220,7 +2172,6 @@
           <t>Module database tập trung</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2256,7 +2207,6 @@
           <t>Dự án RESTful API chạy được nộp qua Git</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2292,7 +2242,6 @@
           <t>ERD mô hình thực thể quan hệ</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2328,7 +2277,6 @@
           <t>Model User &amp; Profile liên kết 1-1</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2364,7 +2312,6 @@
           <t>Model Category &amp; Product liên kết 1-N</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2400,7 +2347,6 @@
           <t>Model liên kết N-N qua bảng trung gian</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2436,7 +2382,6 @@
           <t>API trả về dữ liệu quan hệ lồng nhau</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2472,7 +2417,6 @@
           <t>API dữ liệu liên kết 1-N chạy tốt</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2508,7 +2452,6 @@
           <t>API gán Tag và lấy Product kèm Tags hoạt động</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2544,7 +2487,6 @@
           <t>Hiểu luồng Login chuẩn</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2580,7 +2522,6 @@
           <t>Hiểu cấu trúc chuỗi JWT Token</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2616,7 +2557,6 @@
           <t>Module băm mật khẩu hoạt động tốt</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2652,7 +2592,6 @@
           <t>API Register bảo mật thông tin mật khẩu</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2688,7 +2627,6 @@
           <t>API Login trả về chuỗi JWT Token hợp lệ</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2724,7 +2662,6 @@
           <t>Mô hình ERD Blog + Auth hoàn thiện</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2760,7 +2697,6 @@
           <t>Hệ thống API Blog bảo mật, phân quyền</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2796,7 +2732,6 @@
           <t>Current User Dependency hoạt động</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2832,7 +2767,6 @@
           <t>API phân quyền theo Role bảo mật</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2868,7 +2802,6 @@
           <t>Middleware cơ bản hoạt động</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2904,7 +2837,6 @@
           <t>CORS Middleware hoạt động chính xác</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2940,7 +2872,6 @@
           <t>Endpoint được bảo vệ bằng JWT</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2976,7 +2907,6 @@
           <t>API cho phép kết nối từ Frontend</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3012,7 +2942,6 @@
           <t>API Form hoạt động</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3048,7 +2977,6 @@
           <t>API Upload nhận file thành công</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3084,7 +3012,6 @@
           <t>Lưu trữ file vào thư mục uploads</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3120,7 +3047,6 @@
           <t>Avatar Upload API hoạt động tốt</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3156,7 +3082,6 @@
           <t>Document Upload API + File Storage System</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3192,7 +3117,6 @@
           <t>Test Project khởi tạo thành công</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3228,7 +3152,6 @@
           <t>Test Case GET chạy pass</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3264,7 +3187,6 @@
           <t>Test Case POST chạy pass</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3300,7 +3222,6 @@
           <t>Test Authentication chạy pass</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3336,7 +3257,6 @@
           <t>Đề xuất đề tài dự án &amp; Danh sách nhóm</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3372,7 +3292,6 @@
           <t>Bản vẽ ERD chi tiết của dự án</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3408,7 +3327,6 @@
           <t>Repository GitHub của dự án có khung thư mục chuẩn</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3444,7 +3362,6 @@
           <t>Database MySQL được khởi tạo đầy đủ bảng</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -3480,7 +3397,6 @@
           <t>Các API nghiệp vụ cốt lõi hoạt động tốt</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3516,7 +3432,6 @@
           <t>Hệ thống API phân quyền bảo mật</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -3552,7 +3467,6 @@
           <t>Tính năng upload ảnh và CORS hoạt động tốt</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -3588,7 +3502,6 @@
           <t>Bộ test cases hoạt động kiểm tra lỗi tự động</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -3624,7 +3537,6 @@
           <t>Mã nguồn sạch sẽ, không lỗi và tối ưu hiệu năng</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -3660,7 +3572,6 @@
           <t>Bộ tài liệu hướng dẫn &amp; Slide báo cáo chuyên nghiệp</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -3696,7 +3607,6 @@
           <t>Đánh giá điểm số và hoàn thành môn học xuất sắc</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>